<commit_message>
data of 260828 (more)
</commit_message>
<xml_diff>
--- a/km_math/km.math.group.v9.xlsx
+++ b/km_math/km.math.group.v9.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">Subject</t>
   </si>
@@ -39,9 +39,6 @@
   </si>
   <si>
     <t xml:space="preserve">Prod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">114-002</t>
   </si>
   <si>
     <t xml:space="preserve">115-003</t>
@@ -448,16 +445,16 @@
         <v>9</v>
       </c>
       <c r="B2" t="n">
-        <v>55</v>
+        <v>165</v>
       </c>
       <c r="C2" t="str">
         <f>=B2/(365.25/12)</f>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F2" t="str">
         <f>=IF(D2="TRUE",1,0)</f>
@@ -477,13 +474,13 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C3" t="str">
         <f>=B3/(365.25/12)</f>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E3" t="str">
         <f>=E2-F2-G2</f>
@@ -506,7 +503,7 @@
         <v>11</v>
       </c>
       <c r="B4" t="n">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C4" t="str">
         <f>=B4/(365.25/12)</f>
@@ -535,13 +532,13 @@
         <v>12</v>
       </c>
       <c r="B5" t="n">
-        <v>172</v>
+        <v>223</v>
       </c>
       <c r="C5" t="str">
         <f>=B5/(365.25/12)</f>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E5" t="str">
         <f>=E4-F4-G4</f>
@@ -564,13 +561,13 @@
         <v>13</v>
       </c>
       <c r="B6" t="n">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C6" t="str">
         <f>=B6/(365.25/12)</f>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" t="str">
         <f>=E5-F5-G5</f>
@@ -593,13 +590,13 @@
         <v>14</v>
       </c>
       <c r="B7" t="n">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="C7" t="str">
         <f>=B7/(365.25/12)</f>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7" t="str">
         <f>=E6-F6-G6</f>
@@ -622,13 +619,13 @@
         <v>15</v>
       </c>
       <c r="B8" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C8" t="str">
         <f>=B8/(365.25/12)</f>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E8" t="str">
         <f>=E7-F7-G7</f>
@@ -642,37 +639,8 @@
       <c r="H8" t="str">
         <f>=(E8-F8)/E8</f>
       </c>
-      <c r="I8" t="str">
+      <c r="I8" s="2" t="str">
         <f>=H8*I7</f>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="n">
-        <v>254</v>
-      </c>
-      <c r="C9" t="str">
-        <f>=B9/(365.25/12)</f>
-      </c>
-      <c r="D9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" t="str">
-        <f>=E8-F8-G8</f>
-      </c>
-      <c r="F9" t="str">
-        <f>=IF(D9="TRUE",1,0)</f>
-      </c>
-      <c r="G9" t="str">
-        <f>=1-F9</f>
-      </c>
-      <c r="H9" t="str">
-        <f>=(E9-F9)/E9</f>
-      </c>
-      <c r="I9" s="2" t="str">
-        <f>=H9*I8</f>
       </c>
     </row>
   </sheetData>

</xml_diff>